<commit_message>
Lenovo BRDA DCG (PDF + XLS): flatten line numbering to a single 1..N sequence
Child/component rows are no longer sub-numbered under their parent
(1.01, 1.02, ...); every emitted line now takes the next number in one
running sequence. Since the sequence no longer encodes the hierarchy,
tests now distinguish parent from child by cost (parents priced > 0,
children dropped to 0). Updated parser tests, regenerated the three
Lenovo goldens, and refreshed the Lenovo format specs.
</commit_message>
<xml_diff>
--- a/samples/outputs/BRDAD010458440_NoCalculation_parsed.xlsx
+++ b/samples/outputs/BRDAD010458440_NoCalculation_parsed.xlsx
@@ -114,7 +114,7 @@
     <x:t>256GB ThinkSystem ST650 V3 3yr Base Warranty</x:t>
   </x:si>
   <x:si>
-    <x:t>1.01</x:t>
+    <x:t>2</x:t>
   </x:si>
   <x:si>
     <x:t>BNW0</x:t>
@@ -123,7 +123,7 @@
     <x:t>ThinkSystem ST650 V3 - 2.5" Chassis Base</x:t>
   </x:si>
   <x:si>
-    <x:t>1.02</x:t>
+    <x:t>3</x:t>
   </x:si>
   <x:si>
     <x:t>BFYE</x:t>
@@ -132,7 +132,7 @@
     <x:t>Operating mode selection for: "Efficiency - Favoring Performance Mode"</x:t>
   </x:si>
   <x:si>
-    <x:t>1.03</x:t>
+    <x:t>4</x:t>
   </x:si>
   <x:si>
     <x:t>BNW2</x:t>
@@ -141,7 +141,7 @@
     <x:t>ThinkSystem ST650 V3 System Board</x:t>
   </x:si>
   <x:si>
-    <x:t>1.04</x:t>
+    <x:t>5</x:t>
   </x:si>
   <x:si>
     <x:t>BL0H</x:t>
@@ -150,7 +150,7 @@
     <x:t>Data Center Environment 25 Degree Celsius / 77 Degree Fahrenheit</x:t>
   </x:si>
   <x:si>
-    <x:t>1.05</x:t>
+    <x:t>6</x:t>
   </x:si>
   <x:si>
     <x:t>BYW4</x:t>
@@ -159,7 +159,7 @@
     <x:t>Intel Xeon Silver 4510 12C 150W 2.4GHz Processor</x:t>
   </x:si>
   <x:si>
-    <x:t>1.06</x:t>
+    <x:t>7</x:t>
   </x:si>
   <x:si>
     <x:t>BNF9</x:t>
@@ -168,7 +168,7 @@
     <x:t>ThinkSystem 64GB TruDDR5 4800MHz (2Rx4) 10x4 RDIMM</x:t>
   </x:si>
   <x:si>
-    <x:t>1.07</x:t>
+    <x:t>8</x:t>
   </x:si>
   <x:si>
     <x:t>5978</x:t>
@@ -177,7 +177,7 @@
     <x:t>Select Storage devices - configured RAID</x:t>
   </x:si>
   <x:si>
-    <x:t>1.08</x:t>
+    <x:t>9</x:t>
   </x:si>
   <x:si>
     <x:t>B8NW</x:t>
@@ -186,7 +186,7 @@
     <x:t>ThinkSystem RAID 940-8i 8GB Flash PCIe Gen4 12Gb Adapter</x:t>
   </x:si>
   <x:si>
-    <x:t>1.09</x:t>
+    <x:t>10</x:t>
   </x:si>
   <x:si>
     <x:t>B9XG</x:t>
@@ -195,7 +195,7 @@
     <x:t>Controller 1 HW RAID Array 1 RAID 10</x:t>
   </x:si>
   <x:si>
-    <x:t>1.10</x:t>
+    <x:t>11</x:t>
   </x:si>
   <x:si>
     <x:t>CABV</x:t>
@@ -204,7 +204,7 @@
     <x:t>ThinkSystem 2.5" VA 1.92TB Read Intensive SAS 24Gb HS SSD</x:t>
   </x:si>
   <x:si>
-    <x:t>1.11</x:t>
+    <x:t>12</x:t>
   </x:si>
   <x:si>
     <x:t>B8LU</x:t>
@@ -213,7 +213,7 @@
     <x:t>ThinkSystem 2U 8x2.5" SAS/SATA Backplane</x:t>
   </x:si>
   <x:si>
-    <x:t>1.12</x:t>
+    <x:t>13</x:t>
   </x:si>
   <x:si>
     <x:t>BNFG</x:t>
@@ -222,7 +222,7 @@
     <x:t>ThinkSystem 750W 230V/115V Platinum Hot-Swap Gen2 Power Supply v3</x:t>
   </x:si>
   <x:si>
-    <x:t>1.13</x:t>
+    <x:t>14</x:t>
   </x:si>
   <x:si>
     <x:t>6400</x:t>
@@ -231,7 +231,7 @@
     <x:t>2.8m, 13A/100-250V, C13 to C14 Jumper Cord</x:t>
   </x:si>
   <x:si>
-    <x:t>1.14</x:t>
+    <x:t>15</x:t>
   </x:si>
   <x:si>
     <x:t>BA5T</x:t>
@@ -240,7 +240,7 @@
     <x:t>ThinkSystem ST650 V2 Performance Fan Kit</x:t>
   </x:si>
   <x:si>
-    <x:t>1.15</x:t>
+    <x:t>16</x:t>
   </x:si>
   <x:si>
     <x:t>BPKR</x:t>
@@ -249,7 +249,7 @@
     <x:t>TPM 2.0</x:t>
   </x:si>
   <x:si>
-    <x:t>1.16</x:t>
+    <x:t>17</x:t>
   </x:si>
   <x:si>
     <x:t>C8WV</x:t>
@@ -258,7 +258,7 @@
     <x:t>ST650/ST658 V3 Laser service indicator</x:t>
   </x:si>
   <x:si>
-    <x:t>1.17</x:t>
+    <x:t>18</x:t>
   </x:si>
   <x:si>
     <x:t>2302</x:t>
@@ -267,7 +267,7 @@
     <x:t>RAID Configuration</x:t>
   </x:si>
   <x:si>
-    <x:t>1.18</x:t>
+    <x:t>19</x:t>
   </x:si>
   <x:si>
     <x:t>BNW3</x:t>
@@ -276,7 +276,7 @@
     <x:t>ThinkSystem ST650 V3 Power PADDLE w/ GPU connect</x:t>
   </x:si>
   <x:si>
-    <x:t>1.19</x:t>
+    <x:t>20</x:t>
   </x:si>
   <x:si>
     <x:t>BRPJ</x:t>
@@ -285,7 +285,7 @@
     <x:t>XCC Platinum</x:t>
   </x:si>
   <x:si>
-    <x:t>1.20</x:t>
+    <x:t>21</x:t>
   </x:si>
   <x:si>
     <x:t>BA12</x:t>
@@ -294,7 +294,7 @@
     <x:t>Controller 1 HW RAID Array 1 HDDs</x:t>
   </x:si>
   <x:si>
-    <x:t>1.21</x:t>
+    <x:t>22</x:t>
   </x:si>
   <x:si>
     <x:t>BNWR</x:t>
@@ -303,7 +303,7 @@
     <x:t>ThinkSystem SR860 V3/ST650 V3 CPU Heatsink</x:t>
   </x:si>
   <x:si>
-    <x:t>1.22</x:t>
+    <x:t>23</x:t>
   </x:si>
   <x:si>
     <x:t>AVEN</x:t>
@@ -312,7 +312,7 @@
     <x:t>ThinkSystem 1x1 2.5" HDD Filler</x:t>
   </x:si>
   <x:si>
-    <x:t>1.23</x:t>
+    <x:t>24</x:t>
   </x:si>
   <x:si>
     <x:t>AVEQ</x:t>
@@ -321,7 +321,7 @@
     <x:t>ThinkSystem 8x1 2.5" HDD Filler</x:t>
   </x:si>
   <x:si>
-    <x:t>1.24</x:t>
+    <x:t>25</x:t>
   </x:si>
   <x:si>
     <x:t>AUNP</x:t>
@@ -330,7 +330,7 @@
     <x:t>ThinkSystem RAID 930/940 SuperCap</x:t>
   </x:si>
   <x:si>
-    <x:t>1.25</x:t>
+    <x:t>26</x:t>
   </x:si>
   <x:si>
     <x:t>BP0L</x:t>
@@ -339,7 +339,7 @@
     <x:t>ThinkSystem ST650 V3 RoT Card w/o PFR</x:t>
   </x:si>
   <x:si>
-    <x:t>1.26</x:t>
+    <x:t>27</x:t>
   </x:si>
   <x:si>
     <x:t>5374CM1</x:t>
@@ -348,7 +348,7 @@
     <x:t>software1 Configuration Instruction</x:t>
   </x:si>
   <x:si>
-    <x:t>2</x:t>
+    <x:t>28</x:t>
   </x:si>
   <x:si>
     <x:t>7S0XCTO5WW</x:t>
@@ -357,7 +357,7 @@
     <x:t>software2 XClarity Controller Platin-FOD</x:t>
   </x:si>
   <x:si>
-    <x:t>2.01</x:t>
+    <x:t>29</x:t>
   </x:si>
   <x:si>
     <x:t>SBCV</x:t>
@@ -366,7 +366,7 @@
     <x:t>Lenovo XClarity XCC2 Platinum Upgrade (FOD)</x:t>
   </x:si>
   <x:si>
-    <x:t>3</x:t>
+    <x:t>30</x:t>
   </x:si>
   <x:si>
     <x:t>5PS7C00099</x:t>
@@ -375,7 +375,7 @@
     <x:t>5Yr KYD Add-On ST650 V3</x:t>
   </x:si>
   <x:si>
-    <x:t>4</x:t>
+    <x:t>31</x:t>
   </x:si>
   <x:si>
     <x:t>5WS7C00090</x:t>
@@ -384,100 +384,100 @@
     <x:t>5Yr Premier 24x7 4Hr Resp ST650 V3</x:t>
   </x:si>
   <x:si>
-    <x:t>5</x:t>
+    <x:t>32</x:t>
   </x:si>
   <x:si>
     <x:t>512GB ThinkSystem ST650 V3 3yr Base Warranty</x:t>
   </x:si>
   <x:si>
-    <x:t>5.01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.04</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.05</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.06</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.07</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.08</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.09</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.13</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.14</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.16</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.17</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.19</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.23</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.24</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.25</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.26</x:t>
-  </x:si>
-  <x:si>
-    <x:t>6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>6.01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8</x:t>
+    <x:t>33</x:t>
+  </x:si>
+  <x:si>
+    <x:t>34</x:t>
+  </x:si>
+  <x:si>
+    <x:t>35</x:t>
+  </x:si>
+  <x:si>
+    <x:t>36</x:t>
+  </x:si>
+  <x:si>
+    <x:t>37</x:t>
+  </x:si>
+  <x:si>
+    <x:t>38</x:t>
+  </x:si>
+  <x:si>
+    <x:t>39</x:t>
+  </x:si>
+  <x:si>
+    <x:t>40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>41</x:t>
+  </x:si>
+  <x:si>
+    <x:t>42</x:t>
+  </x:si>
+  <x:si>
+    <x:t>43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>44</x:t>
+  </x:si>
+  <x:si>
+    <x:t>45</x:t>
+  </x:si>
+  <x:si>
+    <x:t>46</x:t>
+  </x:si>
+  <x:si>
+    <x:t>47</x:t>
+  </x:si>
+  <x:si>
+    <x:t>48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>49</x:t>
+  </x:si>
+  <x:si>
+    <x:t>50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>51</x:t>
+  </x:si>
+  <x:si>
+    <x:t>52</x:t>
+  </x:si>
+  <x:si>
+    <x:t>53</x:t>
+  </x:si>
+  <x:si>
+    <x:t>54</x:t>
+  </x:si>
+  <x:si>
+    <x:t>55</x:t>
+  </x:si>
+  <x:si>
+    <x:t>56</x:t>
+  </x:si>
+  <x:si>
+    <x:t>57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>58</x:t>
+  </x:si>
+  <x:si>
+    <x:t>59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>60</x:t>
+  </x:si>
+  <x:si>
+    <x:t>61</x:t>
+  </x:si>
+  <x:si>
+    <x:t>62</x:t>
   </x:si>
   <x:si>
     <x:t>*</x:t>

</xml_diff>